<commit_message>
CAR Varones mobiliario: verificación por texto con etiquetas anidadas en bloques; proyector E7 = 4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_varones/METRADO_EQUIPAMIENTO_Y_MOBILIARIO_CAR_VARONES.xlsx
+++ b/entregables_varones/METRADO_EQUIPAMIENTO_Y_MOBILIARIO_CAR_VARONES.xlsx
@@ -6261,22 +6261,18 @@
           <t>und</t>
         </is>
       </c>
-      <c r="G73" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="H73" s="15" t="n">
-        <v>0</v>
+      <c r="G73" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H73" s="13" t="n">
+        <v>1</v>
       </c>
       <c r="I73" s="14" t="inlineStr">
         <is>
           <t>E7</t>
         </is>
       </c>
-      <c r="J73" s="16" t="inlineStr">
-        <is>
-          <t>El cuadro del tópico repite el de la sala de reuniones (proyector y 10 sillas); en la planta de E-01 hay 2 proyectores (nutrición y sala de reuniones) y 38 sillas M07, no 41.</t>
-        </is>
-      </c>
+      <c r="J73" s="14" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
@@ -6322,7 +6318,7 @@
       </c>
       <c r="J74" s="16" t="inlineStr">
         <is>
-          <t>Ídem: se ajusta el tópico para que E-01 sume las 38 sillas M07 dibujadas.</t>
+          <t>El cuadro del tópico repite las 10 sillas de la sala de reuniones; se ajusta para que E-01 sume las 38 sillas M07 rotuladas en la planta, no 41. El proyector E7 del tópico sí está rotulado.</t>
         </is>
       </c>
     </row>
@@ -16241,7 +16237,7 @@
         <v>43</v>
       </c>
       <c r="E16" s="13" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="F16" s="15">
         <f>'RESUMEN'!E19</f>
@@ -16272,32 +16268,28 @@
           <t>PROYECTOR MULTIMEDIA</t>
         </is>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="C17" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>4</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="15">
+        <v>4</v>
+      </c>
+      <c r="F17" s="13">
         <f>'RESUMEN'!E20</f>
         <v/>
       </c>
-      <c r="G17" s="15">
+      <c r="G17" s="13">
         <f>IF(ISNUMBER(C17),F17-C17,F17)</f>
         <v/>
       </c>
-      <c r="H17" s="17">
+      <c r="H17" s="10">
         <f>IF(G17=0,"conforme","corregir")</f>
         <v/>
       </c>
-      <c r="I17" s="14" t="inlineStr">
-        <is>
-          <t>El metrado original dice 4; el plano da 3. El cuadro del tópico repite el de la sala de reuniones (proyector y 10 sillas); en la planta de E-01 hay 2 proyectores (nutrición y sala de reuniones) y 38 sillas M07, no 41.</t>
-        </is>
-      </c>
+      <c r="I17" s="14" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -16655,7 +16647,7 @@
       </c>
       <c r="I27" s="14" t="inlineStr">
         <is>
-          <t>El metrado original dice 52; el plano da 80. Ídem: se ajusta el tópico para que E-01 sume las 38 sillas M07 dibujadas.</t>
+          <t>El metrado original dice 52; el plano da 80. El cuadro del tópico repite las 10 sillas de la sala de reuniones; se ajusta para que E-01 sume las 38 sillas M07 rotuladas en la planta, no 41. El proyector E7 del tópico sí está rotulado.</t>
         </is>
       </c>
     </row>
@@ -16711,7 +16703,7 @@
         <v>2</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F29" s="13">
         <f>'RESUMEN'!E33</f>
@@ -17849,7 +17841,7 @@
         <v>2</v>
       </c>
       <c r="E61" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F61" s="13">
         <f>'RESUMEN'!E65</f>
@@ -19677,7 +19669,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>El cuadro del tópico repite el de la sala de reuniones: proyector multimedia y 10 sillas.</t>
+          <t>El cuadro del tópico repite las 10 sillas de la sala de reuniones; la planta de E-01 rotula 38 sillas M07 en total, no 41.</t>
         </is>
       </c>
     </row>
@@ -19762,12 +19754,12 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Lámina MB-04, MB-05, MB-01</t>
+          <t>Lámina MB-07</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Sin etiqueta en planta pero sí en su cuadro: las 5 computadoras E6 del salón de estudios (E-04 y E-05) y el rack M13 y la pizarra M69 de la sala de reuniones (E-01); se mantienen.</t>
+          <t>El cuadro del taller de arte pone 1 mueble para mochilas (M56); en planta hay 5.</t>
         </is>
       </c>
     </row>
@@ -19777,12 +19769,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Lámina MB-07</t>
+          <t>Lámina MB-06</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>El cuadro del taller de arte pone 1 mueble para mochilas (M56); en planta hay 5.</t>
+          <t>En el salón de psicomotricidad de E-06 hay 10 cojines cuadrados (K78) dibujados y solo 7 rotulados; se metran los 10 del cuadro.</t>
         </is>
       </c>
     </row>

</xml_diff>